<commit_message>
Progress on LCI choices
</commit_message>
<xml_diff>
--- a/data/LCIs/Lai_2025/Graphite_LCIs_BW_Final_v1.xlsx
+++ b/data/LCIs/Lai_2025/Graphite_LCIs_BW_Final_v1.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="178" documentId="8_{4E3DD59C-3AFA-4D66-BAD6-4D8B482B0214}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0FE8171B-4DE3-4F15-97E4-E0BCC54C54EB}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Note" sheetId="1" r:id="rId1"/>
@@ -6140,12 +6140,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d78c010b-218d-4be4-b2d9-423b1f51aae5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="adc0c41a-12c1-4165-8422-5f5ca88e9f6a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6372,20 +6374,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d78c010b-218d-4be4-b2d9-423b1f51aae5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="adc0c41a-12c1-4165-8422-5f5ca88e9f6a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC223732-7A84-4201-81E0-F4F10B7197AE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3B5D110D-E837-4E58-A07A-E5D7A5B90784}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d78c010b-218d-4be4-b2d9-423b1f51aae5"/>
+    <ds:schemaRef ds:uri="adc0c41a-12c1-4165-8422-5f5ca88e9f6a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -6410,12 +6413,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3B5D110D-E837-4E58-A07A-E5D7A5B90784}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC223732-7A84-4201-81E0-F4F10B7197AE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d78c010b-218d-4be4-b2d9-423b1f51aae5"/>
-    <ds:schemaRef ds:uri="adc0c41a-12c1-4165-8422-5f5ca88e9f6a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>